<commit_message>
working toward driving static loads with LPG--intermediary tests don't work
</commit_message>
<xml_diff>
--- a/tests/ExcelLoadData/TieredLoads_Testing2.xlsx
+++ b/tests/ExcelLoadData/TieredLoads_Testing2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dlvilla\TEMP\TEB\tests\ExcelLoadData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09F9D48-0A4C-47EC-82D0-EFA02CD65425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7C7081-4F6B-4D6C-A23B-D0C8941ED9DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385" xr2:uid="{1F2B6D78-A821-4296-99B9-3A0B6B938907}"/>
+    <workbookView xWindow="4620" yWindow="3420" windowWidth="21600" windowHeight="11385" firstSheet="11" activeTab="14" xr2:uid="{1F2B6D78-A821-4296-99B9-3A0B6B938907}"/>
   </bookViews>
   <sheets>
     <sheet name="StaticElectricLoads" sheetId="1" r:id="rId1"/>
@@ -3827,31 +3827,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{B6E24FE8-171F-4DD9-85AE-EFE65DD5B312}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Villa, Daniel L:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-This comes from 00_ANEJO D.2-Plano-2053-calleCorta-LaPolilla-1un.pdf</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A8" authorId="0" shapeId="0" xr:uid="{503197ED-A21E-4811-8261-3F9E58AEA05B}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{503197ED-A21E-4811-8261-3F9E58AEA05B}">
       <text>
         <r>
           <rPr>
@@ -3875,31 +3851,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A9" authorId="0" shapeId="0" xr:uid="{77CCC27B-5F09-40D8-8D27-B1C1C568B3F5}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Villa, Daniel L:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-This comes from 00_ANEJO D.2-Plano-2053-calleCorta-LaPolilla-1un.pdf</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{DB2A58B4-501A-4078-8B7B-6A2B3EC9A3CD}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{DB2A58B4-501A-4078-8B7B-6A2B3EC9A3CD}">
       <text>
         <r>
           <rPr>
@@ -3923,36 +3875,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{AEEC4A21-16AE-4A3D-A191-83F1114AAC35}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Villa, Daniel L:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-This comes from 00_ANEJO D.2-Plano-2053-calleCorta-LaPolilla-1un.pdf</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="159">
   <si>
     <t>Tier 1</t>
   </si>
@@ -60635,7 +60563,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9025A5CD-2B5D-4B93-BC08-61D2C05FA2C5}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.85546875" bestFit="1" customWidth="1"/>
@@ -60675,73 +60603,49 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>116</v>
-      </c>
-      <c r="B11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>117</v>
-      </c>
-      <c r="B12" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>117</v>
-      </c>
-      <c r="B13" t="s">
         <v>105</v>
       </c>
     </row>
@@ -62613,6 +62517,7 @@
     <col min="10" max="11" width="29.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="30" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>

</xml_diff>